<commit_message>
Add enriched blog post metadata and author profile template
- Enrich blog post metadata: extract Author, Publication Date, and
  Reading Time into the metadata block during import
- Add author-profile template with import script, author-bio parser,
  and foc-author-cleanup transformer for contributor pages
- Add author-bio block (JS + CSS) with responsive layout, circular
  avatar, bio text, and social links
- Update page-templates.json with author-profile template definition

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-blog-post.report.xlsx
+++ b/tools/importer/reports/import-blog-post.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,30 @@
     <t>url</t>
   </si>
   <si>
+    <t>contributor/grant-smith.report.json</t>
+  </si>
+  <si>
+    <t>["author-bio"]</t>
+  </si>
+  <si>
+    <t>contributor/grant-smith</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>author-profile</t>
+  </si>
+  <si>
+    <t>2026-03-20T01:11:02.446Z</t>
+  </si>
+  <si>
+    <t>Grant Smith, Author at The Future of Commerce</t>
+  </si>
+  <si>
+    <t>https://www.the-future-of-commerce.com/contributor/grant-smith/</t>
+  </si>
+  <si>
     <t>2025/05/08/how-sales-ai-helps-in-tough-markets.report.json</t>
   </si>
   <si>
@@ -46,13 +70,10 @@
     <t>2025/05/08/how-sales-ai-helps-in-tough-markets</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>blog-post</t>
   </si>
   <si>
-    <t>2026-03-19T22:26:55.433Z</t>
+    <t>2026-03-20T01:15:51.749Z</t>
   </si>
   <si>
     <t>How sales AI helps organizations grow despite shifting markets</t>
@@ -447,12 +468,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
@@ -509,6 +530,32 @@
         <v>15</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>